<commit_message>
added new data for AVP and Policia
</commit_message>
<xml_diff>
--- a/data/Administracion_de_viviendas_publicas/administracion_vivienda_publica.xlsx
+++ b/data/Administracion_de_viviendas_publicas/administracion_vivienda_publica.xlsx
@@ -1,29 +1,29 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="4" rupBuild="29822"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="4" rupBuild="30026"/>
   <workbookPr defaultThemeVersion="124226"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\gnper\Documents\ViolenciaGeneroPR\data\Administracion_de_viviendas_publicas\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{ADB3DF75-B431-483D-A04A-3AE320C90442}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B6A77D68-B72F-4B8F-9E32-B9E8BADD34A3}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-96" yWindow="0" windowWidth="11712" windowHeight="13056" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="11424" yWindow="0" windowWidth="11712" windowHeight="13056" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="viviendasPublicas_porViolenci" sheetId="1" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">viviendasPublicas_porViolenci!$A$1:$D$181</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">viviendasPublicas_porViolenci!$A$1:$D$199</definedName>
   </definedNames>
   <calcPr calcId="124519"/>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="504" uniqueCount="23">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="544" uniqueCount="23">
   <si>
     <t>Año</t>
   </si>
@@ -447,7 +447,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:G181"/>
+  <dimension ref="A1:G201"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="2" max="2" width="9.88671875" bestFit="1" customWidth="1"/>
@@ -736,36 +736,36 @@
       </c>
     </row>
     <row r="20" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="A20" t="s">
+      <c r="A20" s="2">
+        <v>2026</v>
+      </c>
+      <c r="B20" t="s">
+        <v>5</v>
+      </c>
+      <c r="C20" t="s">
+        <v>6</v>
+      </c>
+      <c r="D20">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="21" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A21" s="2">
+        <v>2026</v>
+      </c>
+      <c r="B21" t="s">
+        <v>5</v>
+      </c>
+      <c r="C21" t="s">
+        <v>7</v>
+      </c>
+      <c r="D21">
         <v>4</v>
-      </c>
-      <c r="B20" t="s">
-        <v>14</v>
-      </c>
-      <c r="C20" t="s">
-        <v>6</v>
-      </c>
-      <c r="D20">
-        <v>21</v>
-      </c>
-    </row>
-    <row r="21" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="A21" t="s">
-        <v>4</v>
-      </c>
-      <c r="B21" t="s">
-        <v>14</v>
-      </c>
-      <c r="C21" t="s">
-        <v>7</v>
-      </c>
-      <c r="D21">
-        <v>5</v>
       </c>
     </row>
     <row r="22" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A22" t="s">
-        <v>8</v>
+        <v>4</v>
       </c>
       <c r="B22" t="s">
         <v>14</v>
@@ -774,12 +774,12 @@
         <v>6</v>
       </c>
       <c r="D22">
-        <v>11</v>
+        <v>21</v>
       </c>
     </row>
     <row r="23" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A23" t="s">
-        <v>8</v>
+        <v>4</v>
       </c>
       <c r="B23" t="s">
         <v>14</v>
@@ -788,12 +788,12 @@
         <v>7</v>
       </c>
       <c r="D23">
-        <v>4</v>
+        <v>5</v>
       </c>
     </row>
     <row r="24" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A24" t="s">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="B24" t="s">
         <v>14</v>
@@ -802,12 +802,12 @@
         <v>6</v>
       </c>
       <c r="D24">
-        <v>7</v>
+        <v>11</v>
       </c>
     </row>
     <row r="25" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A25" t="s">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="B25" t="s">
         <v>14</v>
@@ -816,12 +816,12 @@
         <v>7</v>
       </c>
       <c r="D25">
-        <v>7</v>
+        <v>4</v>
       </c>
     </row>
     <row r="26" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A26" t="s">
-        <v>10</v>
+        <v>9</v>
       </c>
       <c r="B26" t="s">
         <v>14</v>
@@ -830,12 +830,12 @@
         <v>6</v>
       </c>
       <c r="D26">
-        <v>8</v>
+        <v>7</v>
       </c>
     </row>
     <row r="27" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A27" t="s">
-        <v>10</v>
+        <v>9</v>
       </c>
       <c r="B27" t="s">
         <v>14</v>
@@ -844,12 +844,12 @@
         <v>7</v>
       </c>
       <c r="D27">
-        <v>3</v>
+        <v>7</v>
       </c>
     </row>
     <row r="28" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A28" t="s">
-        <v>11</v>
+        <v>10</v>
       </c>
       <c r="B28" t="s">
         <v>14</v>
@@ -858,12 +858,12 @@
         <v>6</v>
       </c>
       <c r="D28">
-        <v>9</v>
+        <v>8</v>
       </c>
     </row>
     <row r="29" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A29" t="s">
-        <v>11</v>
+        <v>10</v>
       </c>
       <c r="B29" t="s">
         <v>14</v>
@@ -872,12 +872,12 @@
         <v>7</v>
       </c>
       <c r="D29">
-        <v>5</v>
+        <v>3</v>
       </c>
     </row>
     <row r="30" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A30" t="s">
-        <v>12</v>
+        <v>11</v>
       </c>
       <c r="B30" t="s">
         <v>14</v>
@@ -886,12 +886,12 @@
         <v>6</v>
       </c>
       <c r="D30">
-        <v>10</v>
+        <v>9</v>
       </c>
     </row>
     <row r="31" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A31" t="s">
-        <v>12</v>
+        <v>11</v>
       </c>
       <c r="B31" t="s">
         <v>14</v>
@@ -900,12 +900,12 @@
         <v>7</v>
       </c>
       <c r="D31">
-        <v>4</v>
+        <v>5</v>
       </c>
     </row>
     <row r="32" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A32" t="s">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="B32" t="s">
         <v>14</v>
@@ -914,12 +914,12 @@
         <v>6</v>
       </c>
       <c r="D32">
-        <v>31</v>
+        <v>10</v>
       </c>
     </row>
     <row r="33" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A33" t="s">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="B33" t="s">
         <v>14</v>
@@ -928,12 +928,12 @@
         <v>7</v>
       </c>
       <c r="D33">
-        <v>9</v>
+        <v>4</v>
       </c>
     </row>
     <row r="34" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="A34" s="2">
-        <v>2024</v>
+      <c r="A34" t="s">
+        <v>13</v>
       </c>
       <c r="B34" t="s">
         <v>14</v>
@@ -942,12 +942,12 @@
         <v>6</v>
       </c>
       <c r="D34">
-        <v>38</v>
+        <v>31</v>
       </c>
     </row>
     <row r="35" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="A35" s="2">
-        <v>2024</v>
+      <c r="A35" t="s">
+        <v>13</v>
       </c>
       <c r="B35" t="s">
         <v>14</v>
@@ -956,12 +956,12 @@
         <v>7</v>
       </c>
       <c r="D35">
-        <v>16</v>
+        <v>9</v>
       </c>
     </row>
     <row r="36" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A36" s="2">
-        <v>2025</v>
+        <v>2024</v>
       </c>
       <c r="B36" t="s">
         <v>14</v>
@@ -970,12 +970,12 @@
         <v>6</v>
       </c>
       <c r="D36">
-        <v>36</v>
+        <v>38</v>
       </c>
     </row>
     <row r="37" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A37" s="2">
-        <v>2025</v>
+        <v>2024</v>
       </c>
       <c r="B37" t="s">
         <v>14</v>
@@ -984,68 +984,68 @@
         <v>7</v>
       </c>
       <c r="D37">
+        <v>16</v>
+      </c>
+    </row>
+    <row r="38" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A38" s="2">
+        <v>2025</v>
+      </c>
+      <c r="B38" t="s">
+        <v>14</v>
+      </c>
+      <c r="C38" t="s">
+        <v>6</v>
+      </c>
+      <c r="D38">
+        <v>36</v>
+      </c>
+    </row>
+    <row r="39" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A39" s="2">
+        <v>2025</v>
+      </c>
+      <c r="B39" t="s">
+        <v>14</v>
+      </c>
+      <c r="C39" t="s">
+        <v>7</v>
+      </c>
+      <c r="D39">
         <v>24</v>
       </c>
     </row>
-    <row r="38" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="A38" t="s">
-        <v>4</v>
-      </c>
-      <c r="B38" t="s">
-        <v>15</v>
-      </c>
-      <c r="C38" t="s">
-        <v>6</v>
-      </c>
-      <c r="D38">
-        <v>18</v>
-      </c>
-    </row>
-    <row r="39" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="A39" t="s">
-        <v>4</v>
-      </c>
-      <c r="B39" t="s">
-        <v>15</v>
-      </c>
-      <c r="C39" t="s">
-        <v>7</v>
-      </c>
-      <c r="D39">
-        <v>3</v>
-      </c>
-    </row>
     <row r="40" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="A40" t="s">
-        <v>8</v>
+      <c r="A40" s="2">
+        <v>2026</v>
       </c>
       <c r="B40" t="s">
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="C40" t="s">
         <v>6</v>
       </c>
       <c r="D40">
+        <v>16</v>
+      </c>
+    </row>
+    <row r="41" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A41" s="2">
+        <v>2026</v>
+      </c>
+      <c r="B41" t="s">
         <v>14</v>
       </c>
-    </row>
-    <row r="41" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="A41" t="s">
-        <v>8</v>
-      </c>
-      <c r="B41" t="s">
-        <v>15</v>
-      </c>
       <c r="C41" t="s">
         <v>7</v>
       </c>
       <c r="D41">
-        <v>2</v>
+        <v>1</v>
       </c>
     </row>
     <row r="42" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A42" t="s">
-        <v>9</v>
+        <v>4</v>
       </c>
       <c r="B42" t="s">
         <v>15</v>
@@ -1054,12 +1054,12 @@
         <v>6</v>
       </c>
       <c r="D42">
-        <v>6</v>
+        <v>18</v>
       </c>
     </row>
     <row r="43" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A43" t="s">
-        <v>9</v>
+        <v>4</v>
       </c>
       <c r="B43" t="s">
         <v>15</v>
@@ -1068,12 +1068,12 @@
         <v>7</v>
       </c>
       <c r="D43">
-        <v>4</v>
+        <v>3</v>
       </c>
     </row>
     <row r="44" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A44" t="s">
-        <v>10</v>
+        <v>8</v>
       </c>
       <c r="B44" t="s">
         <v>15</v>
@@ -1082,12 +1082,12 @@
         <v>6</v>
       </c>
       <c r="D44">
-        <v>9</v>
+        <v>14</v>
       </c>
     </row>
     <row r="45" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A45" t="s">
-        <v>10</v>
+        <v>8</v>
       </c>
       <c r="B45" t="s">
         <v>15</v>
@@ -1096,12 +1096,12 @@
         <v>7</v>
       </c>
       <c r="D45">
-        <v>3</v>
+        <v>2</v>
       </c>
     </row>
     <row r="46" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A46" t="s">
-        <v>11</v>
+        <v>9</v>
       </c>
       <c r="B46" t="s">
         <v>15</v>
@@ -1110,12 +1110,12 @@
         <v>6</v>
       </c>
       <c r="D46">
-        <v>13</v>
+        <v>6</v>
       </c>
     </row>
     <row r="47" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A47" t="s">
-        <v>11</v>
+        <v>9</v>
       </c>
       <c r="B47" t="s">
         <v>15</v>
@@ -1129,7 +1129,7 @@
     </row>
     <row r="48" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A48" t="s">
-        <v>12</v>
+        <v>10</v>
       </c>
       <c r="B48" t="s">
         <v>15</v>
@@ -1138,12 +1138,12 @@
         <v>6</v>
       </c>
       <c r="D48">
-        <v>13</v>
+        <v>9</v>
       </c>
     </row>
     <row r="49" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A49" t="s">
-        <v>12</v>
+        <v>10</v>
       </c>
       <c r="B49" t="s">
         <v>15</v>
@@ -1152,12 +1152,12 @@
         <v>7</v>
       </c>
       <c r="D49">
-        <v>9</v>
+        <v>3</v>
       </c>
     </row>
     <row r="50" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A50" t="s">
-        <v>13</v>
+        <v>11</v>
       </c>
       <c r="B50" t="s">
         <v>15</v>
@@ -1166,12 +1166,12 @@
         <v>6</v>
       </c>
       <c r="D50">
-        <v>58</v>
+        <v>13</v>
       </c>
     </row>
     <row r="51" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A51" t="s">
-        <v>13</v>
+        <v>11</v>
       </c>
       <c r="B51" t="s">
         <v>15</v>
@@ -1180,12 +1180,12 @@
         <v>7</v>
       </c>
       <c r="D51">
-        <v>10</v>
+        <v>4</v>
       </c>
     </row>
     <row r="52" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="A52" s="2">
-        <v>2024</v>
+      <c r="A52" t="s">
+        <v>12</v>
       </c>
       <c r="B52" t="s">
         <v>15</v>
@@ -1194,12 +1194,12 @@
         <v>6</v>
       </c>
       <c r="D52">
-        <v>73</v>
+        <v>13</v>
       </c>
     </row>
     <row r="53" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="A53" s="2">
-        <v>2024</v>
+      <c r="A53" t="s">
+        <v>12</v>
       </c>
       <c r="B53" t="s">
         <v>15</v>
@@ -1208,12 +1208,12 @@
         <v>7</v>
       </c>
       <c r="D53">
-        <v>25</v>
+        <v>9</v>
       </c>
     </row>
     <row r="54" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="A54" s="2">
-        <v>2025</v>
+      <c r="A54" t="s">
+        <v>13</v>
       </c>
       <c r="B54" t="s">
         <v>15</v>
@@ -1222,12 +1222,12 @@
         <v>6</v>
       </c>
       <c r="D54">
-        <v>48</v>
+        <v>58</v>
       </c>
     </row>
     <row r="55" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="A55" s="2">
-        <v>2025</v>
+      <c r="A55" t="s">
+        <v>13</v>
       </c>
       <c r="B55" t="s">
         <v>15</v>
@@ -1236,96 +1236,96 @@
         <v>7</v>
       </c>
       <c r="D55">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="56" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A56" s="2">
+        <v>2024</v>
+      </c>
+      <c r="B56" t="s">
+        <v>15</v>
+      </c>
+      <c r="C56" t="s">
+        <v>6</v>
+      </c>
+      <c r="D56">
+        <v>73</v>
+      </c>
+    </row>
+    <row r="57" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A57" s="2">
+        <v>2024</v>
+      </c>
+      <c r="B57" t="s">
+        <v>15</v>
+      </c>
+      <c r="C57" t="s">
+        <v>7</v>
+      </c>
+      <c r="D57">
+        <v>25</v>
+      </c>
+    </row>
+    <row r="58" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A58" s="2">
+        <v>2025</v>
+      </c>
+      <c r="B58" t="s">
+        <v>15</v>
+      </c>
+      <c r="C58" t="s">
+        <v>6</v>
+      </c>
+      <c r="D58">
+        <v>48</v>
+      </c>
+    </row>
+    <row r="59" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A59" s="2">
+        <v>2025</v>
+      </c>
+      <c r="B59" t="s">
+        <v>15</v>
+      </c>
+      <c r="C59" t="s">
+        <v>7</v>
+      </c>
+      <c r="D59">
         <v>24</v>
       </c>
     </row>
-    <row r="56" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="A56" t="s">
-        <v>4</v>
-      </c>
-      <c r="B56" t="s">
-        <v>16</v>
-      </c>
-      <c r="C56" t="s">
-        <v>6</v>
-      </c>
-      <c r="D56">
-        <v>53</v>
-      </c>
-    </row>
-    <row r="57" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="A57" t="s">
-        <v>4</v>
-      </c>
-      <c r="B57" t="s">
-        <v>16</v>
-      </c>
-      <c r="C57" t="s">
-        <v>7</v>
-      </c>
-      <c r="D57">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="58" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="A58" t="s">
-        <v>8</v>
-      </c>
-      <c r="B58" t="s">
-        <v>16</v>
-      </c>
-      <c r="C58" t="s">
-        <v>6</v>
-      </c>
-      <c r="D58">
-        <v>28</v>
-      </c>
-    </row>
-    <row r="59" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="A59" t="s">
-        <v>8</v>
-      </c>
-      <c r="B59" t="s">
-        <v>16</v>
-      </c>
-      <c r="C59" t="s">
-        <v>7</v>
-      </c>
-      <c r="D59">
-        <v>5</v>
-      </c>
-    </row>
     <row r="60" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="A60" t="s">
-        <v>9</v>
+      <c r="A60" s="2">
+        <v>2026</v>
       </c>
       <c r="B60" t="s">
-        <v>16</v>
+        <v>15</v>
       </c>
       <c r="C60" t="s">
         <v>6</v>
       </c>
       <c r="D60">
+        <v>24</v>
+      </c>
+    </row>
+    <row r="61" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A61" s="2">
+        <v>2026</v>
+      </c>
+      <c r="B61" t="s">
         <v>15</v>
       </c>
-    </row>
-    <row r="61" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="A61" t="s">
-        <v>9</v>
-      </c>
-      <c r="B61" t="s">
-        <v>16</v>
-      </c>
       <c r="C61" t="s">
         <v>7</v>
       </c>
       <c r="D61">
-        <v>3</v>
+        <v>6</v>
       </c>
     </row>
     <row r="62" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A62" t="s">
-        <v>10</v>
+        <v>4</v>
       </c>
       <c r="B62" t="s">
         <v>16</v>
@@ -1334,12 +1334,12 @@
         <v>6</v>
       </c>
       <c r="D62">
-        <v>12</v>
+        <v>53</v>
       </c>
     </row>
     <row r="63" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A63" t="s">
-        <v>10</v>
+        <v>4</v>
       </c>
       <c r="B63" t="s">
         <v>16</v>
@@ -1348,12 +1348,12 @@
         <v>7</v>
       </c>
       <c r="D63">
-        <v>3</v>
+        <v>1</v>
       </c>
     </row>
     <row r="64" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A64" t="s">
-        <v>11</v>
+        <v>8</v>
       </c>
       <c r="B64" t="s">
         <v>16</v>
@@ -1367,7 +1367,7 @@
     </row>
     <row r="65" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A65" t="s">
-        <v>11</v>
+        <v>8</v>
       </c>
       <c r="B65" t="s">
         <v>16</v>
@@ -1376,12 +1376,12 @@
         <v>7</v>
       </c>
       <c r="D65">
-        <v>4</v>
+        <v>5</v>
       </c>
     </row>
     <row r="66" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A66" t="s">
-        <v>12</v>
+        <v>9</v>
       </c>
       <c r="B66" t="s">
         <v>16</v>
@@ -1390,12 +1390,12 @@
         <v>6</v>
       </c>
       <c r="D66">
-        <v>24</v>
+        <v>15</v>
       </c>
     </row>
     <row r="67" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A67" t="s">
-        <v>12</v>
+        <v>9</v>
       </c>
       <c r="B67" t="s">
         <v>16</v>
@@ -1404,12 +1404,12 @@
         <v>7</v>
       </c>
       <c r="D67">
-        <v>4</v>
+        <v>3</v>
       </c>
     </row>
     <row r="68" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A68" t="s">
-        <v>13</v>
+        <v>10</v>
       </c>
       <c r="B68" t="s">
         <v>16</v>
@@ -1418,12 +1418,12 @@
         <v>6</v>
       </c>
       <c r="D68">
-        <v>20</v>
+        <v>12</v>
       </c>
     </row>
     <row r="69" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A69" t="s">
-        <v>13</v>
+        <v>10</v>
       </c>
       <c r="B69" t="s">
         <v>16</v>
@@ -1432,12 +1432,12 @@
         <v>7</v>
       </c>
       <c r="D69">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="70" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A70" t="s">
         <v>11</v>
-      </c>
-    </row>
-    <row r="70" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="A70" s="2">
-        <v>2024</v>
       </c>
       <c r="B70" t="s">
         <v>16</v>
@@ -1446,12 +1446,12 @@
         <v>6</v>
       </c>
       <c r="D70">
-        <v>27</v>
+        <v>28</v>
       </c>
     </row>
     <row r="71" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="A71" s="2">
-        <v>2024</v>
+      <c r="A71" t="s">
+        <v>11</v>
       </c>
       <c r="B71" t="s">
         <v>16</v>
@@ -1460,12 +1460,12 @@
         <v>7</v>
       </c>
       <c r="D71">
-        <v>2</v>
+        <v>4</v>
       </c>
     </row>
     <row r="72" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="A72" s="2">
-        <v>2025</v>
+      <c r="A72" t="s">
+        <v>12</v>
       </c>
       <c r="B72" t="s">
         <v>16</v>
@@ -1474,12 +1474,12 @@
         <v>6</v>
       </c>
       <c r="D72">
-        <v>27</v>
+        <v>24</v>
       </c>
     </row>
     <row r="73" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="A73" s="2">
-        <v>2025</v>
+      <c r="A73" t="s">
+        <v>12</v>
       </c>
       <c r="B73" t="s">
         <v>16</v>
@@ -1488,124 +1488,124 @@
         <v>7</v>
       </c>
       <c r="D73">
-        <v>20</v>
+        <v>4</v>
       </c>
     </row>
     <row r="74" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A74" t="s">
-        <v>4</v>
+        <v>13</v>
       </c>
       <c r="B74" t="s">
-        <v>17</v>
+        <v>16</v>
       </c>
       <c r="C74" t="s">
         <v>6</v>
       </c>
       <c r="D74">
-        <v>102</v>
+        <v>20</v>
       </c>
     </row>
     <row r="75" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A75" t="s">
-        <v>4</v>
+        <v>13</v>
       </c>
       <c r="B75" t="s">
-        <v>17</v>
+        <v>16</v>
       </c>
       <c r="C75" t="s">
         <v>7</v>
       </c>
       <c r="D75">
-        <v>6</v>
+        <v>11</v>
       </c>
     </row>
     <row r="76" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="A76" t="s">
-        <v>8</v>
+      <c r="A76" s="2">
+        <v>2024</v>
       </c>
       <c r="B76" t="s">
-        <v>17</v>
+        <v>16</v>
       </c>
       <c r="C76" t="s">
         <v>6</v>
       </c>
       <c r="D76">
-        <v>48</v>
+        <v>27</v>
       </c>
     </row>
     <row r="77" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="A77" t="s">
-        <v>8</v>
+      <c r="A77" s="2">
+        <v>2024</v>
       </c>
       <c r="B77" t="s">
-        <v>17</v>
+        <v>16</v>
       </c>
       <c r="C77" t="s">
         <v>7</v>
       </c>
       <c r="D77">
-        <v>3</v>
+        <v>2</v>
       </c>
     </row>
     <row r="78" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="A78" t="s">
+      <c r="A78" s="2">
+        <v>2025</v>
+      </c>
+      <c r="B78" t="s">
+        <v>16</v>
+      </c>
+      <c r="C78" t="s">
+        <v>6</v>
+      </c>
+      <c r="D78">
+        <v>27</v>
+      </c>
+    </row>
+    <row r="79" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A79" s="2">
+        <v>2025</v>
+      </c>
+      <c r="B79" t="s">
+        <v>16</v>
+      </c>
+      <c r="C79" t="s">
+        <v>7</v>
+      </c>
+      <c r="D79">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="80" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A80" s="2">
+        <v>2026</v>
+      </c>
+      <c r="B80" t="s">
+        <v>16</v>
+      </c>
+      <c r="C80" t="s">
+        <v>6</v>
+      </c>
+      <c r="D80">
         <v>9</v>
       </c>
-      <c r="B78" t="s">
-        <v>17</v>
-      </c>
-      <c r="C78" t="s">
-        <v>6</v>
-      </c>
-      <c r="D78">
-        <v>23</v>
-      </c>
-    </row>
-    <row r="79" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="A79" t="s">
-        <v>9</v>
-      </c>
-      <c r="B79" t="s">
-        <v>17</v>
-      </c>
-      <c r="C79" t="s">
-        <v>7</v>
-      </c>
-      <c r="D79">
-        <v>4</v>
-      </c>
-    </row>
-    <row r="80" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="A80" t="s">
-        <v>10</v>
-      </c>
-      <c r="B80" t="s">
-        <v>17</v>
-      </c>
-      <c r="C80" t="s">
-        <v>6</v>
-      </c>
-      <c r="D80">
-        <v>19</v>
-      </c>
     </row>
     <row r="81" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="A81" t="s">
-        <v>10</v>
+      <c r="A81" s="2">
+        <v>2026</v>
       </c>
       <c r="B81" t="s">
-        <v>17</v>
+        <v>16</v>
       </c>
       <c r="C81" t="s">
         <v>7</v>
       </c>
       <c r="D81">
-        <v>5</v>
+        <v>1</v>
       </c>
     </row>
     <row r="82" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A82" t="s">
-        <v>11</v>
+        <v>4</v>
       </c>
       <c r="B82" t="s">
         <v>17</v>
@@ -1614,12 +1614,12 @@
         <v>6</v>
       </c>
       <c r="D82">
-        <v>26</v>
+        <v>102</v>
       </c>
     </row>
     <row r="83" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A83" t="s">
-        <v>11</v>
+        <v>4</v>
       </c>
       <c r="B83" t="s">
         <v>17</v>
@@ -1628,12 +1628,12 @@
         <v>7</v>
       </c>
       <c r="D83">
-        <v>7</v>
+        <v>6</v>
       </c>
     </row>
     <row r="84" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A84" t="s">
-        <v>12</v>
+        <v>8</v>
       </c>
       <c r="B84" t="s">
         <v>17</v>
@@ -1642,12 +1642,12 @@
         <v>6</v>
       </c>
       <c r="D84">
-        <v>53</v>
+        <v>48</v>
       </c>
     </row>
     <row r="85" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A85" t="s">
-        <v>12</v>
+        <v>8</v>
       </c>
       <c r="B85" t="s">
         <v>17</v>
@@ -1656,12 +1656,12 @@
         <v>7</v>
       </c>
       <c r="D85">
-        <v>9</v>
+        <v>3</v>
       </c>
     </row>
     <row r="86" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A86" t="s">
-        <v>13</v>
+        <v>9</v>
       </c>
       <c r="B86" t="s">
         <v>17</v>
@@ -1670,12 +1670,12 @@
         <v>6</v>
       </c>
       <c r="D86">
-        <v>62</v>
+        <v>23</v>
       </c>
     </row>
     <row r="87" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A87" t="s">
-        <v>13</v>
+        <v>9</v>
       </c>
       <c r="B87" t="s">
         <v>17</v>
@@ -1684,12 +1684,12 @@
         <v>7</v>
       </c>
       <c r="D87">
-        <v>12</v>
+        <v>4</v>
       </c>
     </row>
     <row r="88" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="A88" s="2">
-        <v>2024</v>
+      <c r="A88" t="s">
+        <v>10</v>
       </c>
       <c r="B88" t="s">
         <v>17</v>
@@ -1698,12 +1698,12 @@
         <v>6</v>
       </c>
       <c r="D88">
-        <v>65</v>
+        <v>19</v>
       </c>
     </row>
     <row r="89" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="A89" s="2">
-        <v>2024</v>
+      <c r="A89" t="s">
+        <v>10</v>
       </c>
       <c r="B89" t="s">
         <v>17</v>
@@ -1712,12 +1712,12 @@
         <v>7</v>
       </c>
       <c r="D89">
-        <v>20</v>
+        <v>5</v>
       </c>
     </row>
     <row r="90" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="A90" s="2">
-        <v>2025</v>
+      <c r="A90" t="s">
+        <v>11</v>
       </c>
       <c r="B90" t="s">
         <v>17</v>
@@ -1726,12 +1726,12 @@
         <v>6</v>
       </c>
       <c r="D90">
-        <v>52</v>
+        <v>26</v>
       </c>
     </row>
     <row r="91" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="A91" s="2">
-        <v>2025</v>
+      <c r="A91" t="s">
+        <v>11</v>
       </c>
       <c r="B91" t="s">
         <v>17</v>
@@ -1740,152 +1740,152 @@
         <v>7</v>
       </c>
       <c r="D91">
-        <v>25</v>
+        <v>7</v>
       </c>
     </row>
     <row r="92" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A92" t="s">
-        <v>4</v>
+        <v>12</v>
       </c>
       <c r="B92" t="s">
-        <v>18</v>
+        <v>17</v>
       </c>
       <c r="C92" t="s">
         <v>6</v>
       </c>
       <c r="D92">
-        <v>8</v>
+        <v>53</v>
       </c>
     </row>
     <row r="93" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A93" t="s">
-        <v>4</v>
+        <v>12</v>
       </c>
       <c r="B93" t="s">
-        <v>18</v>
+        <v>17</v>
       </c>
       <c r="C93" t="s">
         <v>7</v>
       </c>
       <c r="D93">
-        <v>0</v>
+        <v>9</v>
       </c>
     </row>
     <row r="94" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A94" t="s">
-        <v>8</v>
+        <v>13</v>
       </c>
       <c r="B94" t="s">
-        <v>18</v>
+        <v>17</v>
       </c>
       <c r="C94" t="s">
         <v>6</v>
       </c>
       <c r="D94">
-        <v>3</v>
+        <v>62</v>
       </c>
     </row>
     <row r="95" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A95" t="s">
-        <v>8</v>
+        <v>13</v>
       </c>
       <c r="B95" t="s">
-        <v>18</v>
+        <v>17</v>
       </c>
       <c r="C95" t="s">
         <v>7</v>
       </c>
       <c r="D95">
-        <v>1</v>
+        <v>12</v>
       </c>
     </row>
     <row r="96" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="A96" t="s">
-        <v>9</v>
+      <c r="A96" s="2">
+        <v>2024</v>
       </c>
       <c r="B96" t="s">
-        <v>18</v>
+        <v>17</v>
       </c>
       <c r="C96" t="s">
         <v>6</v>
       </c>
       <c r="D96">
-        <v>7</v>
+        <v>65</v>
       </c>
     </row>
     <row r="97" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="A97" t="s">
-        <v>9</v>
+      <c r="A97" s="2">
+        <v>2024</v>
       </c>
       <c r="B97" t="s">
-        <v>18</v>
+        <v>17</v>
       </c>
       <c r="C97" t="s">
         <v>7</v>
       </c>
       <c r="D97">
-        <v>2</v>
+        <v>20</v>
       </c>
     </row>
     <row r="98" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="A98" t="s">
-        <v>10</v>
+      <c r="A98" s="2">
+        <v>2025</v>
       </c>
       <c r="B98" t="s">
-        <v>18</v>
+        <v>17</v>
       </c>
       <c r="C98" t="s">
         <v>6</v>
       </c>
       <c r="D98">
-        <v>0</v>
+        <v>52</v>
       </c>
     </row>
     <row r="99" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="A99" t="s">
-        <v>10</v>
+      <c r="A99" s="2">
+        <v>2025</v>
       </c>
       <c r="B99" t="s">
-        <v>18</v>
+        <v>17</v>
       </c>
       <c r="C99" t="s">
         <v>7</v>
       </c>
       <c r="D99">
-        <v>0</v>
+        <v>25</v>
       </c>
     </row>
     <row r="100" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="A100" t="s">
-        <v>11</v>
+      <c r="A100" s="2">
+        <v>2026</v>
       </c>
       <c r="B100" t="s">
-        <v>18</v>
+        <v>17</v>
       </c>
       <c r="C100" t="s">
         <v>6</v>
       </c>
       <c r="D100">
-        <v>0</v>
+        <v>36</v>
       </c>
     </row>
     <row r="101" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="A101" t="s">
-        <v>11</v>
+      <c r="A101" s="2">
+        <v>2026</v>
       </c>
       <c r="B101" t="s">
-        <v>18</v>
+        <v>17</v>
       </c>
       <c r="C101" t="s">
         <v>7</v>
       </c>
       <c r="D101">
-        <v>1</v>
+        <v>6</v>
       </c>
     </row>
     <row r="102" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A102" t="s">
-        <v>12</v>
+        <v>4</v>
       </c>
       <c r="B102" t="s">
         <v>18</v>
@@ -1894,12 +1894,12 @@
         <v>6</v>
       </c>
       <c r="D102">
-        <v>11</v>
+        <v>8</v>
       </c>
     </row>
     <row r="103" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A103" t="s">
-        <v>12</v>
+        <v>4</v>
       </c>
       <c r="B103" t="s">
         <v>18</v>
@@ -1908,12 +1908,12 @@
         <v>7</v>
       </c>
       <c r="D103">
-        <v>2</v>
+        <v>0</v>
       </c>
     </row>
     <row r="104" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A104" t="s">
-        <v>13</v>
+        <v>8</v>
       </c>
       <c r="B104" t="s">
         <v>18</v>
@@ -1922,12 +1922,12 @@
         <v>6</v>
       </c>
       <c r="D104">
-        <v>35</v>
+        <v>3</v>
       </c>
     </row>
     <row r="105" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A105" t="s">
-        <v>13</v>
+        <v>8</v>
       </c>
       <c r="B105" t="s">
         <v>18</v>
@@ -1936,12 +1936,12 @@
         <v>7</v>
       </c>
       <c r="D105">
-        <v>4</v>
+        <v>1</v>
       </c>
     </row>
     <row r="106" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="A106" s="2">
-        <v>2024</v>
+      <c r="A106" t="s">
+        <v>9</v>
       </c>
       <c r="B106" t="s">
         <v>18</v>
@@ -1950,12 +1950,12 @@
         <v>6</v>
       </c>
       <c r="D106">
-        <v>39</v>
+        <v>7</v>
       </c>
     </row>
     <row r="107" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="A107" s="2">
-        <v>2024</v>
+      <c r="A107" t="s">
+        <v>9</v>
       </c>
       <c r="B107" t="s">
         <v>18</v>
@@ -1964,12 +1964,12 @@
         <v>7</v>
       </c>
       <c r="D107">
-        <v>15</v>
+        <v>2</v>
       </c>
     </row>
     <row r="108" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="A108" s="2">
-        <v>2025</v>
+      <c r="A108" t="s">
+        <v>10</v>
       </c>
       <c r="B108" t="s">
         <v>18</v>
@@ -1978,12 +1978,12 @@
         <v>6</v>
       </c>
       <c r="D108">
-        <v>26</v>
+        <v>0</v>
       </c>
     </row>
     <row r="109" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="A109" s="2">
-        <v>2025</v>
+      <c r="A109" t="s">
+        <v>10</v>
       </c>
       <c r="B109" t="s">
         <v>18</v>
@@ -1992,29 +1992,29 @@
         <v>7</v>
       </c>
       <c r="D109">
-        <v>18</v>
+        <v>0</v>
       </c>
     </row>
     <row r="110" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A110" t="s">
-        <v>4</v>
+        <v>11</v>
       </c>
       <c r="B110" t="s">
-        <v>19</v>
+        <v>18</v>
       </c>
       <c r="C110" t="s">
         <v>6</v>
       </c>
       <c r="D110">
-        <v>7</v>
+        <v>0</v>
       </c>
     </row>
     <row r="111" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A111" t="s">
-        <v>4</v>
+        <v>11</v>
       </c>
       <c r="B111" t="s">
-        <v>19</v>
+        <v>18</v>
       </c>
       <c r="C111" t="s">
         <v>7</v>
@@ -2025,147 +2025,147 @@
     </row>
     <row r="112" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A112" t="s">
-        <v>8</v>
+        <v>12</v>
       </c>
       <c r="B112" t="s">
-        <v>19</v>
+        <v>18</v>
       </c>
       <c r="C112" t="s">
         <v>6</v>
       </c>
       <c r="D112">
-        <v>17</v>
+        <v>11</v>
       </c>
     </row>
     <row r="113" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A113" t="s">
-        <v>8</v>
+        <v>12</v>
       </c>
       <c r="B113" t="s">
-        <v>19</v>
+        <v>18</v>
       </c>
       <c r="C113" t="s">
         <v>7</v>
       </c>
       <c r="D113">
-        <v>1</v>
+        <v>2</v>
       </c>
     </row>
     <row r="114" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A114" t="s">
-        <v>9</v>
+        <v>13</v>
       </c>
       <c r="B114" t="s">
-        <v>19</v>
+        <v>18</v>
       </c>
       <c r="C114" t="s">
         <v>6</v>
       </c>
       <c r="D114">
-        <v>12</v>
+        <v>35</v>
       </c>
     </row>
     <row r="115" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A115" t="s">
-        <v>9</v>
+        <v>13</v>
       </c>
       <c r="B115" t="s">
-        <v>19</v>
+        <v>18</v>
       </c>
       <c r="C115" t="s">
         <v>7</v>
       </c>
       <c r="D115">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="116" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A116" s="2">
+        <v>2024</v>
+      </c>
+      <c r="B116" t="s">
+        <v>18</v>
+      </c>
+      <c r="C116" t="s">
+        <v>6</v>
+      </c>
+      <c r="D116">
+        <v>39</v>
+      </c>
+    </row>
+    <row r="117" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A117" s="2">
+        <v>2024</v>
+      </c>
+      <c r="B117" t="s">
+        <v>18</v>
+      </c>
+      <c r="C117" t="s">
+        <v>7</v>
+      </c>
+      <c r="D117">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="118" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A118" s="2">
+        <v>2025</v>
+      </c>
+      <c r="B118" t="s">
+        <v>18</v>
+      </c>
+      <c r="C118" t="s">
+        <v>6</v>
+      </c>
+      <c r="D118">
+        <v>26</v>
+      </c>
+    </row>
+    <row r="119" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A119" s="2">
+        <v>2025</v>
+      </c>
+      <c r="B119" t="s">
+        <v>18</v>
+      </c>
+      <c r="C119" t="s">
+        <v>7</v>
+      </c>
+      <c r="D119">
+        <v>18</v>
+      </c>
+    </row>
+    <row r="120" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A120" s="2">
+        <v>2026</v>
+      </c>
+      <c r="B120" t="s">
+        <v>18</v>
+      </c>
+      <c r="C120" t="s">
+        <v>6</v>
+      </c>
+      <c r="D120">
+        <v>14</v>
+      </c>
+    </row>
+    <row r="121" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A121" s="2">
+        <v>2026</v>
+      </c>
+      <c r="B121" t="s">
+        <v>18</v>
+      </c>
+      <c r="C121" t="s">
+        <v>7</v>
+      </c>
+      <c r="D121">
         <v>3</v>
-      </c>
-    </row>
-    <row r="116" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="A116" t="s">
-        <v>10</v>
-      </c>
-      <c r="B116" t="s">
-        <v>19</v>
-      </c>
-      <c r="C116" t="s">
-        <v>6</v>
-      </c>
-      <c r="D116">
-        <v>11</v>
-      </c>
-    </row>
-    <row r="117" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="A117" t="s">
-        <v>10</v>
-      </c>
-      <c r="B117" t="s">
-        <v>19</v>
-      </c>
-      <c r="C117" t="s">
-        <v>7</v>
-      </c>
-      <c r="D117">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="118" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="A118" t="s">
-        <v>11</v>
-      </c>
-      <c r="B118" t="s">
-        <v>19</v>
-      </c>
-      <c r="C118" t="s">
-        <v>6</v>
-      </c>
-      <c r="D118">
-        <v>14</v>
-      </c>
-    </row>
-    <row r="119" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="A119" t="s">
-        <v>11</v>
-      </c>
-      <c r="B119" t="s">
-        <v>19</v>
-      </c>
-      <c r="C119" t="s">
-        <v>7</v>
-      </c>
-      <c r="D119">
-        <v>2</v>
-      </c>
-    </row>
-    <row r="120" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="A120" t="s">
-        <v>12</v>
-      </c>
-      <c r="B120" t="s">
-        <v>19</v>
-      </c>
-      <c r="C120" t="s">
-        <v>6</v>
-      </c>
-      <c r="D120">
-        <v>7</v>
-      </c>
-    </row>
-    <row r="121" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="A121" t="s">
-        <v>12</v>
-      </c>
-      <c r="B121" t="s">
-        <v>19</v>
-      </c>
-      <c r="C121" t="s">
-        <v>7</v>
-      </c>
-      <c r="D121">
-        <v>6</v>
       </c>
     </row>
     <row r="122" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A122" t="s">
-        <v>13</v>
+        <v>4</v>
       </c>
       <c r="B122" t="s">
         <v>19</v>
@@ -2174,12 +2174,12 @@
         <v>6</v>
       </c>
       <c r="D122">
-        <v>8</v>
+        <v>7</v>
       </c>
     </row>
     <row r="123" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A123" t="s">
-        <v>13</v>
+        <v>4</v>
       </c>
       <c r="B123" t="s">
         <v>19</v>
@@ -2188,12 +2188,12 @@
         <v>7</v>
       </c>
       <c r="D123">
-        <v>10</v>
+        <v>1</v>
       </c>
     </row>
     <row r="124" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="A124" s="2">
-        <v>2024</v>
+      <c r="A124" t="s">
+        <v>8</v>
       </c>
       <c r="B124" t="s">
         <v>19</v>
@@ -2202,12 +2202,12 @@
         <v>6</v>
       </c>
       <c r="D124">
-        <v>19</v>
+        <v>17</v>
       </c>
     </row>
     <row r="125" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="A125" s="2">
-        <v>2024</v>
+      <c r="A125" t="s">
+        <v>8</v>
       </c>
       <c r="B125" t="s">
         <v>19</v>
@@ -2216,12 +2216,12 @@
         <v>7</v>
       </c>
       <c r="D125">
-        <v>12</v>
+        <v>1</v>
       </c>
     </row>
     <row r="126" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="A126" s="2">
-        <v>2025</v>
+      <c r="A126" t="s">
+        <v>9</v>
       </c>
       <c r="B126" t="s">
         <v>19</v>
@@ -2230,12 +2230,12 @@
         <v>6</v>
       </c>
       <c r="D126">
-        <v>20</v>
+        <v>12</v>
       </c>
     </row>
     <row r="127" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="A127" s="2">
-        <v>2025</v>
+      <c r="A127" t="s">
+        <v>9</v>
       </c>
       <c r="B127" t="s">
         <v>19</v>
@@ -2244,57 +2244,57 @@
         <v>7</v>
       </c>
       <c r="D127">
-        <v>15</v>
-      </c>
-    </row>
-    <row r="128" spans="1:4" ht="12.6" customHeight="1" x14ac:dyDescent="0.3">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="128" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A128" t="s">
-        <v>4</v>
+        <v>10</v>
       </c>
       <c r="B128" t="s">
-        <v>20</v>
+        <v>19</v>
       </c>
       <c r="C128" t="s">
         <v>6</v>
       </c>
       <c r="D128">
-        <v>5</v>
+        <v>11</v>
       </c>
     </row>
     <row r="129" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A129" t="s">
-        <v>4</v>
+        <v>10</v>
       </c>
       <c r="B129" t="s">
-        <v>20</v>
+        <v>19</v>
       </c>
       <c r="C129" t="s">
         <v>7</v>
       </c>
       <c r="D129">
-        <v>3</v>
+        <v>1</v>
       </c>
     </row>
     <row r="130" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A130" t="s">
-        <v>8</v>
+        <v>11</v>
       </c>
       <c r="B130" t="s">
-        <v>20</v>
+        <v>19</v>
       </c>
       <c r="C130" t="s">
         <v>6</v>
       </c>
       <c r="D130">
-        <v>2</v>
+        <v>14</v>
       </c>
     </row>
     <row r="131" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A131" t="s">
-        <v>8</v>
+        <v>11</v>
       </c>
       <c r="B131" t="s">
-        <v>20</v>
+        <v>19</v>
       </c>
       <c r="C131" t="s">
         <v>7</v>
@@ -2305,147 +2305,147 @@
     </row>
     <row r="132" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A132" t="s">
-        <v>9</v>
+        <v>12</v>
       </c>
       <c r="B132" t="s">
-        <v>20</v>
+        <v>19</v>
       </c>
       <c r="C132" t="s">
         <v>6</v>
       </c>
       <c r="D132">
-        <v>5</v>
+        <v>7</v>
       </c>
     </row>
     <row r="133" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A133" t="s">
-        <v>9</v>
+        <v>12</v>
       </c>
       <c r="B133" t="s">
-        <v>20</v>
+        <v>19</v>
       </c>
       <c r="C133" t="s">
         <v>7</v>
       </c>
       <c r="D133">
-        <v>1</v>
+        <v>6</v>
       </c>
     </row>
     <row r="134" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A134" t="s">
-        <v>10</v>
+        <v>13</v>
       </c>
       <c r="B134" t="s">
-        <v>20</v>
+        <v>19</v>
       </c>
       <c r="C134" t="s">
         <v>6</v>
       </c>
       <c r="D134">
-        <v>1</v>
+        <v>8</v>
       </c>
     </row>
     <row r="135" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A135" t="s">
+        <v>13</v>
+      </c>
+      <c r="B135" t="s">
+        <v>19</v>
+      </c>
+      <c r="C135" t="s">
+        <v>7</v>
+      </c>
+      <c r="D135">
         <v>10</v>
       </c>
-      <c r="B135" t="s">
+    </row>
+    <row r="136" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A136" s="2">
+        <v>2024</v>
+      </c>
+      <c r="B136" t="s">
+        <v>19</v>
+      </c>
+      <c r="C136" t="s">
+        <v>6</v>
+      </c>
+      <c r="D136">
+        <v>19</v>
+      </c>
+    </row>
+    <row r="137" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A137" s="2">
+        <v>2024</v>
+      </c>
+      <c r="B137" t="s">
+        <v>19</v>
+      </c>
+      <c r="C137" t="s">
+        <v>7</v>
+      </c>
+      <c r="D137">
+        <v>12</v>
+      </c>
+    </row>
+    <row r="138" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A138" s="2">
+        <v>2025</v>
+      </c>
+      <c r="B138" t="s">
+        <v>19</v>
+      </c>
+      <c r="C138" t="s">
+        <v>6</v>
+      </c>
+      <c r="D138">
         <v>20</v>
       </c>
-      <c r="C135" t="s">
-        <v>7</v>
-      </c>
-      <c r="D135">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="136" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="A136" t="s">
-        <v>11</v>
-      </c>
-      <c r="B136" t="s">
-        <v>20</v>
-      </c>
-      <c r="C136" t="s">
-        <v>6</v>
-      </c>
-      <c r="D136">
-        <v>3</v>
-      </c>
-    </row>
-    <row r="137" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="A137" t="s">
-        <v>11</v>
-      </c>
-      <c r="B137" t="s">
-        <v>20</v>
-      </c>
-      <c r="C137" t="s">
-        <v>7</v>
-      </c>
-      <c r="D137">
-        <v>3</v>
-      </c>
-    </row>
-    <row r="138" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="A138" t="s">
-        <v>12</v>
-      </c>
-      <c r="B138" t="s">
-        <v>20</v>
-      </c>
-      <c r="C138" t="s">
-        <v>6</v>
-      </c>
-      <c r="D138">
-        <v>7</v>
-      </c>
     </row>
     <row r="139" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="A139" t="s">
-        <v>12</v>
+      <c r="A139" s="2">
+        <v>2025</v>
       </c>
       <c r="B139" t="s">
-        <v>20</v>
+        <v>19</v>
       </c>
       <c r="C139" t="s">
         <v>7</v>
       </c>
       <c r="D139">
-        <v>3</v>
+        <v>15</v>
       </c>
     </row>
     <row r="140" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="A140" t="s">
-        <v>13</v>
+      <c r="A140" s="2">
+        <v>2026</v>
       </c>
       <c r="B140" t="s">
-        <v>20</v>
+        <v>19</v>
       </c>
       <c r="C140" t="s">
         <v>6</v>
       </c>
       <c r="D140">
-        <v>7</v>
+        <v>2</v>
       </c>
     </row>
     <row r="141" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="A141" t="s">
-        <v>13</v>
+      <c r="A141" s="2">
+        <v>2026</v>
       </c>
       <c r="B141" t="s">
-        <v>20</v>
+        <v>19</v>
       </c>
       <c r="C141" t="s">
         <v>7</v>
       </c>
       <c r="D141">
-        <v>6</v>
-      </c>
-    </row>
-    <row r="142" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="A142" s="2">
-        <v>2024</v>
+        <v>2</v>
+      </c>
+    </row>
+    <row r="142" spans="1:4" ht="12.6" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A142" t="s">
+        <v>4</v>
       </c>
       <c r="B142" t="s">
         <v>20</v>
@@ -2454,12 +2454,12 @@
         <v>6</v>
       </c>
       <c r="D142">
-        <v>19</v>
+        <v>5</v>
       </c>
     </row>
     <row r="143" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="A143" s="2">
-        <v>2024</v>
+      <c r="A143" t="s">
+        <v>4</v>
       </c>
       <c r="B143" t="s">
         <v>20</v>
@@ -2468,12 +2468,12 @@
         <v>7</v>
       </c>
       <c r="D143">
-        <v>11</v>
+        <v>3</v>
       </c>
     </row>
     <row r="144" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="A144" s="2">
-        <v>2025</v>
+      <c r="A144" t="s">
+        <v>8</v>
       </c>
       <c r="B144" t="s">
         <v>20</v>
@@ -2482,12 +2482,12 @@
         <v>6</v>
       </c>
       <c r="D144">
-        <v>14</v>
+        <v>2</v>
       </c>
     </row>
     <row r="145" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="A145" s="2">
-        <v>2025</v>
+      <c r="A145" t="s">
+        <v>8</v>
       </c>
       <c r="B145" t="s">
         <v>20</v>
@@ -2496,169 +2496,169 @@
         <v>7</v>
       </c>
       <c r="D145">
-        <v>13</v>
+        <v>2</v>
       </c>
     </row>
     <row r="146" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A146" t="s">
-        <v>4</v>
+        <v>9</v>
       </c>
       <c r="B146" t="s">
-        <v>21</v>
+        <v>20</v>
       </c>
       <c r="C146" t="s">
         <v>6</v>
       </c>
       <c r="D146">
-        <v>19</v>
+        <v>5</v>
       </c>
     </row>
     <row r="147" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A147" t="s">
-        <v>4</v>
+        <v>9</v>
       </c>
       <c r="B147" t="s">
-        <v>21</v>
+        <v>20</v>
       </c>
       <c r="C147" t="s">
         <v>7</v>
       </c>
       <c r="D147">
-        <v>6</v>
+        <v>1</v>
       </c>
     </row>
     <row r="148" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A148" t="s">
-        <v>8</v>
+        <v>10</v>
       </c>
       <c r="B148" t="s">
-        <v>21</v>
+        <v>20</v>
       </c>
       <c r="C148" t="s">
         <v>6</v>
       </c>
       <c r="D148">
-        <v>12</v>
+        <v>1</v>
       </c>
     </row>
     <row r="149" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A149" t="s">
-        <v>8</v>
+        <v>10</v>
       </c>
       <c r="B149" t="s">
-        <v>21</v>
+        <v>20</v>
       </c>
       <c r="C149" t="s">
         <v>7</v>
       </c>
       <c r="D149">
-        <v>9</v>
+        <v>1</v>
       </c>
     </row>
     <row r="150" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A150" t="s">
-        <v>9</v>
+        <v>11</v>
       </c>
       <c r="B150" t="s">
-        <v>21</v>
+        <v>20</v>
       </c>
       <c r="C150" t="s">
         <v>6</v>
       </c>
       <c r="D150">
-        <v>7</v>
+        <v>3</v>
       </c>
     </row>
     <row r="151" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A151" t="s">
-        <v>9</v>
+        <v>11</v>
       </c>
       <c r="B151" t="s">
-        <v>21</v>
+        <v>20</v>
       </c>
       <c r="C151" t="s">
         <v>7</v>
       </c>
       <c r="D151">
-        <v>9</v>
+        <v>3</v>
       </c>
     </row>
     <row r="152" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A152" t="s">
-        <v>10</v>
+        <v>12</v>
       </c>
       <c r="B152" t="s">
-        <v>21</v>
+        <v>20</v>
       </c>
       <c r="C152" t="s">
         <v>6</v>
       </c>
       <c r="D152">
-        <v>8</v>
+        <v>7</v>
       </c>
     </row>
     <row r="153" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A153" t="s">
-        <v>10</v>
+        <v>12</v>
       </c>
       <c r="B153" t="s">
-        <v>21</v>
+        <v>20</v>
       </c>
       <c r="C153" t="s">
         <v>7</v>
       </c>
       <c r="D153">
-        <v>0</v>
+        <v>3</v>
       </c>
     </row>
     <row r="154" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A154" t="s">
-        <v>11</v>
+        <v>13</v>
       </c>
       <c r="B154" t="s">
-        <v>21</v>
+        <v>20</v>
       </c>
       <c r="C154" t="s">
         <v>6</v>
       </c>
       <c r="D154">
-        <v>24</v>
+        <v>7</v>
       </c>
     </row>
     <row r="155" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A155" t="s">
-        <v>11</v>
+        <v>13</v>
       </c>
       <c r="B155" t="s">
-        <v>21</v>
+        <v>20</v>
       </c>
       <c r="C155" t="s">
         <v>7</v>
       </c>
       <c r="D155">
-        <v>10</v>
+        <v>6</v>
       </c>
     </row>
     <row r="156" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="A156" t="s">
-        <v>12</v>
+      <c r="A156" s="2">
+        <v>2024</v>
       </c>
       <c r="B156" t="s">
-        <v>21</v>
+        <v>20</v>
       </c>
       <c r="C156" t="s">
         <v>6</v>
       </c>
       <c r="D156">
+        <v>19</v>
+      </c>
+    </row>
+    <row r="157" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A157" s="2">
+        <v>2024</v>
+      </c>
+      <c r="B157" t="s">
         <v>20</v>
-      </c>
-    </row>
-    <row r="157" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="A157" t="s">
-        <v>12</v>
-      </c>
-      <c r="B157" t="s">
-        <v>21</v>
       </c>
       <c r="C157" t="s">
         <v>7</v>
@@ -2668,64 +2668,64 @@
       </c>
     </row>
     <row r="158" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="A158" t="s">
+      <c r="A158" s="2">
+        <v>2025</v>
+      </c>
+      <c r="B158" t="s">
+        <v>20</v>
+      </c>
+      <c r="C158" t="s">
+        <v>6</v>
+      </c>
+      <c r="D158">
+        <v>14</v>
+      </c>
+    </row>
+    <row r="159" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A159" s="2">
+        <v>2025</v>
+      </c>
+      <c r="B159" t="s">
+        <v>20</v>
+      </c>
+      <c r="C159" t="s">
+        <v>7</v>
+      </c>
+      <c r="D159">
         <v>13</v>
-      </c>
-      <c r="B158" t="s">
-        <v>21</v>
-      </c>
-      <c r="C158" t="s">
-        <v>6</v>
-      </c>
-      <c r="D158">
-        <v>33</v>
-      </c>
-    </row>
-    <row r="159" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="A159" t="s">
-        <v>13</v>
-      </c>
-      <c r="B159" t="s">
-        <v>21</v>
-      </c>
-      <c r="C159" t="s">
-        <v>7</v>
-      </c>
-      <c r="D159">
-        <v>21</v>
       </c>
     </row>
     <row r="160" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A160" s="2">
-        <v>2024</v>
+        <v>2026</v>
       </c>
       <c r="B160" t="s">
-        <v>21</v>
+        <v>20</v>
       </c>
       <c r="C160" t="s">
         <v>6</v>
       </c>
       <c r="D160">
-        <v>60</v>
+        <v>13</v>
       </c>
     </row>
     <row r="161" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A161" s="2">
-        <v>2024</v>
+        <v>2026</v>
       </c>
       <c r="B161" t="s">
-        <v>21</v>
+        <v>20</v>
       </c>
       <c r="C161" t="s">
         <v>7</v>
       </c>
       <c r="D161">
-        <v>37</v>
+        <v>6</v>
       </c>
     </row>
     <row r="162" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="A162" s="2">
-        <v>2025</v>
+      <c r="A162" t="s">
+        <v>4</v>
       </c>
       <c r="B162" t="s">
         <v>21</v>
@@ -2734,12 +2734,12 @@
         <v>6</v>
       </c>
       <c r="D162">
-        <v>48</v>
+        <v>19</v>
       </c>
     </row>
     <row r="163" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="A163" s="2">
-        <v>2025</v>
+      <c r="A163" t="s">
+        <v>4</v>
       </c>
       <c r="B163" t="s">
         <v>21</v>
@@ -2748,127 +2748,127 @@
         <v>7</v>
       </c>
       <c r="D163">
-        <v>33</v>
+        <v>6</v>
       </c>
     </row>
     <row r="164" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A164" t="s">
-        <v>4</v>
+        <v>8</v>
       </c>
       <c r="B164" t="s">
-        <v>22</v>
+        <v>21</v>
       </c>
       <c r="C164" t="s">
         <v>6</v>
       </c>
       <c r="D164">
-        <v>14</v>
+        <v>12</v>
       </c>
     </row>
     <row r="165" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A165" t="s">
-        <v>4</v>
+        <v>8</v>
       </c>
       <c r="B165" t="s">
-        <v>22</v>
+        <v>21</v>
       </c>
       <c r="C165" t="s">
         <v>7</v>
       </c>
       <c r="D165">
-        <v>5</v>
+        <v>9</v>
       </c>
     </row>
     <row r="166" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A166" t="s">
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="B166" t="s">
-        <v>22</v>
+        <v>21</v>
       </c>
       <c r="C166" t="s">
         <v>6</v>
       </c>
       <c r="D166">
-        <v>16</v>
+        <v>7</v>
       </c>
     </row>
     <row r="167" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A167" t="s">
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="B167" t="s">
-        <v>22</v>
+        <v>21</v>
       </c>
       <c r="C167" t="s">
         <v>7</v>
       </c>
       <c r="D167">
-        <v>3</v>
+        <v>9</v>
       </c>
     </row>
     <row r="168" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A168" t="s">
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="B168" t="s">
-        <v>22</v>
+        <v>21</v>
       </c>
       <c r="C168" t="s">
         <v>6</v>
       </c>
       <c r="D168">
-        <v>11</v>
+        <v>8</v>
       </c>
     </row>
     <row r="169" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A169" t="s">
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="B169" t="s">
-        <v>22</v>
+        <v>21</v>
       </c>
       <c r="C169" t="s">
         <v>7</v>
       </c>
       <c r="D169">
-        <v>13</v>
+        <v>0</v>
       </c>
     </row>
     <row r="170" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A170" t="s">
-        <v>10</v>
+        <v>11</v>
       </c>
       <c r="B170" t="s">
-        <v>22</v>
+        <v>21</v>
       </c>
       <c r="C170" t="s">
         <v>6</v>
       </c>
       <c r="D170">
-        <v>7</v>
+        <v>24</v>
       </c>
     </row>
     <row r="171" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A171" t="s">
+        <v>11</v>
+      </c>
+      <c r="B171" t="s">
+        <v>21</v>
+      </c>
+      <c r="C171" t="s">
+        <v>7</v>
+      </c>
+      <c r="D171">
         <v>10</v>
-      </c>
-      <c r="B171" t="s">
-        <v>22</v>
-      </c>
-      <c r="C171" t="s">
-        <v>7</v>
-      </c>
-      <c r="D171">
-        <v>0</v>
       </c>
     </row>
     <row r="172" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A172" t="s">
-        <v>11</v>
+        <v>12</v>
       </c>
       <c r="B172" t="s">
-        <v>22</v>
+        <v>21</v>
       </c>
       <c r="C172" t="s">
         <v>6</v>
@@ -2879,10 +2879,10 @@
     </row>
     <row r="173" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A173" t="s">
-        <v>11</v>
+        <v>12</v>
       </c>
       <c r="B173" t="s">
-        <v>22</v>
+        <v>21</v>
       </c>
       <c r="C173" t="s">
         <v>7</v>
@@ -2893,24 +2893,24 @@
     </row>
     <row r="174" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A174" t="s">
-        <v>12</v>
+        <v>13</v>
       </c>
       <c r="B174" t="s">
-        <v>22</v>
+        <v>21</v>
       </c>
       <c r="C174" t="s">
         <v>6</v>
       </c>
       <c r="D174">
-        <v>27</v>
+        <v>33</v>
       </c>
     </row>
     <row r="175" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A175" t="s">
-        <v>12</v>
+        <v>13</v>
       </c>
       <c r="B175" t="s">
-        <v>22</v>
+        <v>21</v>
       </c>
       <c r="C175" t="s">
         <v>7</v>
@@ -2920,87 +2920,367 @@
       </c>
     </row>
     <row r="176" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="A176" t="s">
-        <v>13</v>
+      <c r="A176" s="2">
+        <v>2024</v>
       </c>
       <c r="B176" t="s">
-        <v>22</v>
+        <v>21</v>
       </c>
       <c r="C176" t="s">
         <v>6</v>
       </c>
       <c r="D176">
-        <v>17</v>
+        <v>60</v>
       </c>
     </row>
     <row r="177" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="A177" t="s">
-        <v>13</v>
+      <c r="A177" s="2">
+        <v>2024</v>
       </c>
       <c r="B177" t="s">
-        <v>22</v>
+        <v>21</v>
       </c>
       <c r="C177" t="s">
         <v>7</v>
       </c>
       <c r="D177">
-        <v>30</v>
+        <v>37</v>
       </c>
     </row>
     <row r="178" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A178" s="2">
-        <v>2024</v>
+        <v>2025</v>
       </c>
       <c r="B178" t="s">
-        <v>22</v>
+        <v>21</v>
       </c>
       <c r="C178" t="s">
         <v>6</v>
       </c>
       <c r="D178">
-        <v>69</v>
+        <v>48</v>
       </c>
     </row>
     <row r="179" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A179" s="2">
-        <v>2024</v>
+        <v>2025</v>
       </c>
       <c r="B179" t="s">
-        <v>22</v>
+        <v>21</v>
       </c>
       <c r="C179" t="s">
         <v>7</v>
       </c>
       <c r="D179">
-        <v>38</v>
+        <v>33</v>
       </c>
     </row>
     <row r="180" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A180" s="2">
-        <v>2025</v>
+        <v>2026</v>
       </c>
       <c r="B180" t="s">
-        <v>22</v>
+        <v>21</v>
       </c>
       <c r="C180" t="s">
         <v>6</v>
       </c>
       <c r="D180">
-        <v>91</v>
+        <v>23</v>
       </c>
     </row>
     <row r="181" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A181" s="2">
+        <v>2026</v>
+      </c>
+      <c r="B181" t="s">
+        <v>21</v>
+      </c>
+      <c r="C181" t="s">
+        <v>7</v>
+      </c>
+      <c r="D181">
+        <v>16</v>
+      </c>
+    </row>
+    <row r="182" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A182" t="s">
+        <v>4</v>
+      </c>
+      <c r="B182" t="s">
+        <v>22</v>
+      </c>
+      <c r="C182" t="s">
+        <v>6</v>
+      </c>
+      <c r="D182">
+        <v>14</v>
+      </c>
+    </row>
+    <row r="183" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A183" t="s">
+        <v>4</v>
+      </c>
+      <c r="B183" t="s">
+        <v>22</v>
+      </c>
+      <c r="C183" t="s">
+        <v>7</v>
+      </c>
+      <c r="D183">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="184" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A184" t="s">
+        <v>8</v>
+      </c>
+      <c r="B184" t="s">
+        <v>22</v>
+      </c>
+      <c r="C184" t="s">
+        <v>6</v>
+      </c>
+      <c r="D184">
+        <v>16</v>
+      </c>
+    </row>
+    <row r="185" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A185" t="s">
+        <v>8</v>
+      </c>
+      <c r="B185" t="s">
+        <v>22</v>
+      </c>
+      <c r="C185" t="s">
+        <v>7</v>
+      </c>
+      <c r="D185">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="186" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A186" t="s">
+        <v>9</v>
+      </c>
+      <c r="B186" t="s">
+        <v>22</v>
+      </c>
+      <c r="C186" t="s">
+        <v>6</v>
+      </c>
+      <c r="D186">
+        <v>11</v>
+      </c>
+    </row>
+    <row r="187" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A187" t="s">
+        <v>9</v>
+      </c>
+      <c r="B187" t="s">
+        <v>22</v>
+      </c>
+      <c r="C187" t="s">
+        <v>7</v>
+      </c>
+      <c r="D187">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="188" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A188" t="s">
+        <v>10</v>
+      </c>
+      <c r="B188" t="s">
+        <v>22</v>
+      </c>
+      <c r="C188" t="s">
+        <v>6</v>
+      </c>
+      <c r="D188">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="189" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A189" t="s">
+        <v>10</v>
+      </c>
+      <c r="B189" t="s">
+        <v>22</v>
+      </c>
+      <c r="C189" t="s">
+        <v>7</v>
+      </c>
+      <c r="D189">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="190" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A190" t="s">
+        <v>11</v>
+      </c>
+      <c r="B190" t="s">
+        <v>22</v>
+      </c>
+      <c r="C190" t="s">
+        <v>6</v>
+      </c>
+      <c r="D190">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="191" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A191" t="s">
+        <v>11</v>
+      </c>
+      <c r="B191" t="s">
+        <v>22</v>
+      </c>
+      <c r="C191" t="s">
+        <v>7</v>
+      </c>
+      <c r="D191">
+        <v>11</v>
+      </c>
+    </row>
+    <row r="192" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A192" t="s">
+        <v>12</v>
+      </c>
+      <c r="B192" t="s">
+        <v>22</v>
+      </c>
+      <c r="C192" t="s">
+        <v>6</v>
+      </c>
+      <c r="D192">
+        <v>27</v>
+      </c>
+    </row>
+    <row r="193" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A193" t="s">
+        <v>12</v>
+      </c>
+      <c r="B193" t="s">
+        <v>22</v>
+      </c>
+      <c r="C193" t="s">
+        <v>7</v>
+      </c>
+      <c r="D193">
+        <v>21</v>
+      </c>
+    </row>
+    <row r="194" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A194" t="s">
+        <v>13</v>
+      </c>
+      <c r="B194" t="s">
+        <v>22</v>
+      </c>
+      <c r="C194" t="s">
+        <v>6</v>
+      </c>
+      <c r="D194">
+        <v>17</v>
+      </c>
+    </row>
+    <row r="195" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A195" t="s">
+        <v>13</v>
+      </c>
+      <c r="B195" t="s">
+        <v>22</v>
+      </c>
+      <c r="C195" t="s">
+        <v>7</v>
+      </c>
+      <c r="D195">
+        <v>30</v>
+      </c>
+    </row>
+    <row r="196" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A196" s="2">
+        <v>2024</v>
+      </c>
+      <c r="B196" t="s">
+        <v>22</v>
+      </c>
+      <c r="C196" t="s">
+        <v>6</v>
+      </c>
+      <c r="D196">
+        <v>69</v>
+      </c>
+    </row>
+    <row r="197" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A197" s="2">
+        <v>2024</v>
+      </c>
+      <c r="B197" t="s">
+        <v>22</v>
+      </c>
+      <c r="C197" t="s">
+        <v>7</v>
+      </c>
+      <c r="D197">
+        <v>38</v>
+      </c>
+    </row>
+    <row r="198" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A198" s="2">
         <v>2025</v>
       </c>
-      <c r="B181" t="s">
+      <c r="B198" t="s">
         <v>22</v>
       </c>
-      <c r="C181" t="s">
-        <v>7</v>
-      </c>
-      <c r="D181">
+      <c r="C198" t="s">
+        <v>6</v>
+      </c>
+      <c r="D198">
+        <v>91</v>
+      </c>
+    </row>
+    <row r="199" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A199" s="2">
+        <v>2025</v>
+      </c>
+      <c r="B199" t="s">
+        <v>22</v>
+      </c>
+      <c r="C199" t="s">
+        <v>7</v>
+      </c>
+      <c r="D199">
         <v>65</v>
+      </c>
+    </row>
+    <row r="200" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A200" s="2">
+        <v>2026</v>
+      </c>
+      <c r="B200" t="s">
+        <v>22</v>
+      </c>
+      <c r="C200" t="s">
+        <v>6</v>
+      </c>
+      <c r="D200">
+        <v>28</v>
+      </c>
+    </row>
+    <row r="201" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A201" s="2">
+        <v>2026</v>
+      </c>
+      <c r="B201" t="s">
+        <v>22</v>
+      </c>
+      <c r="C201" t="s">
+        <v>7</v>
+      </c>
+      <c r="D201">
+        <v>21</v>
       </c>
     </row>
   </sheetData>

</xml_diff>